<commit_message>
Regen: stage R_materials_final done
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/research_materials/01_training/training_runs.xlsx
+++ b/research_materials/01_training/training_runs.xlsx
@@ -464,7 +464,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Built: 2026-10-06 23:35 by src/build_research_materials.py</t>
+          <t>Built: 2026-10-07 02:02 by src/build_research_materials.py</t>
         </is>
       </c>
     </row>
@@ -1645,11 +1645,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
     <col width="21" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
   </cols>
@@ -1874,6 +1874,28 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>regen</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>deployment_variants_matching_base</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07 02:01:19</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>merged AWQ/RTN/GGUF on the dequantized base need the dequantized checkpoint + llm-compressor + a further judge/MiniCheck swap; resume: see STATUS.md</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>